<commit_message>
Phase 3v12 audit fixes: _xlfn prefixes + tblStateRates as real table
Pre-open audit caught two issues that would have caused #NAME? errors:

1. All 6 LAMBDAs lacked the _xlfn. / _xlfn._xlws. prefixes that Excel
   requires for modern functions (LAMBDA, LET, FILTER, XLOOKUP) when
   stored in defined names. Patched all instances.

2. State rates section was added in v10 as a named range, not a real
   Excel table. TAX_STATE's structured refs (tblStateRates[State],
   tblStateRates[Top_Marginal_Rate]) would have failed to resolve.
   Converted Tax_Ref!B618:F669 to a real Table named tblStateRates.

Final audit confirms all structured references across all 6 LAMBDAs
resolve to existing tables and columns.
</commit_message>
<xml_diff>
--- a/docs/Master_Pivot_Framework_v5_phase3v12_CC.xlsx
+++ b/docs/Master_Pivot_Framework_v5_phase3v12_CC.xlsx
@@ -145,12 +145,12 @@
     <definedName name="States">Dropdown_Lists!$I$4:$I$54</definedName>
     <definedName name="tblStateRates">Tax_Ref!$B$619:$F$669</definedName>
     <definedName name="PTET_States">Tax_Ref!$B$619:$D$669</definedName>
-    <definedName name="TAX_ORD">LAMBDA(taxable_income,year,fs,LET(rows,FILTER(tblBrackets_FIT,(tblBrackets_FIT[Year]=year)*(tblBrackets_FIT[FilingStatus]=fs)*(tblBrackets_FIT[Lower]&lt;=taxable_income)*(tblBrackets_FIT[Upper]&gt;taxable_income)),lower,INDEX(rows,1,3),rate,INDEX(rows,1,5),add_to,INDEX(rows,1,6),MAX(0,(taxable_income-lower)*rate+add_to)))</definedName>
-    <definedName name="TAX_CG">LAMBDA(cg_amount,taxable_income,year,fs,LET(rows,FILTER(tblBrackets_LTCG,(tblBrackets_LTCG[Year]=year)*(tblBrackets_LTCG[FilingStatus]=fs)*(tblBrackets_LTCG[Lower]&lt;=taxable_income)*(tblBrackets_LTCG[Upper]&gt;taxable_income)),rate,INDEX(rows,1,5),cg_amount*rate))</definedName>
-    <definedName name="TAX_NIIT">LAMBDA(net_inv_income,magi,fs,year,LET(threshold,INDEX(FILTER(tblThresholds[Value],(tblThresholds[Item]="NIIT_Threshold")*(tblThresholds[Year]=year)*(tblThresholds[FilingStatus]=fs)),1),rate,0.038,MAX(0,MIN(net_inv_income,magi-threshold))*rate))</definedName>
-    <definedName name="TAX_SE">LAMBDA(se_net_earnings,year,LET(se_base,se_net_earnings*0.9235,ss_cap,INDEX(FILTER(tblThresholds[Value],(tblThresholds[Item]="SS_Wage_Base")*(tblThresholds[Year]=year)),1),ss_tax,MIN(se_base,ss_cap)*0.124,medi_tax,se_base*0.029,ss_tax+medi_tax))</definedName>
-    <definedName name="STD_DED">LAMBDA(year,fs,INDEX(FILTER(tblStdDed[Amount],(tblStdDed[Year]=year)*(tblStdDed[FilingStatus]=fs)),1))</definedName>
-    <definedName name="TAX_STATE">LAMBDA(taxable_income,state,taxable_income*XLOOKUP(state,tblStateRates[State],tblStateRates[Top_Marginal_Rate],0))</definedName>
+    <definedName name="TAX_ORD">_xlfn.LAMBDA(taxable_income,year,fs,_xlfn.LET(rows,_xlfn._xlws.FILTER(tblBrackets_FIT,(tblBrackets_FIT[Year]=year)*(tblBrackets_FIT[FilingStatus]=fs)*(tblBrackets_FIT[Lower]&lt;=taxable_income)*(tblBrackets_FIT[Upper]&gt;taxable_income)),lower,INDEX(rows,1,3),rate,INDEX(rows,1,5),add_to,INDEX(rows,1,6),MAX(0,(taxable_income-lower)*rate+add_to)))</definedName>
+    <definedName name="TAX_CG">_xlfn.LAMBDA(cg_amount,taxable_income,year,fs,_xlfn.LET(rows,_xlfn._xlws.FILTER(tblBrackets_LTCG,(tblBrackets_LTCG[Year]=year)*(tblBrackets_LTCG[FilingStatus]=fs)*(tblBrackets_LTCG[Lower]&lt;=taxable_income)*(tblBrackets_LTCG[Upper]&gt;taxable_income)),rate,INDEX(rows,1,5),cg_amount*rate))</definedName>
+    <definedName name="TAX_NIIT">_xlfn.LAMBDA(net_inv_income,magi,fs,year,_xlfn.LET(threshold,INDEX(_xlfn._xlws.FILTER(tblThresholds[Value],(tblThresholds[Item]="NIIT_Threshold")*(tblThresholds[Year]=year)*(tblThresholds[FilingStatus]=fs)),1),rate,0.038,MAX(0,MIN(net_inv_income,magi-threshold))*rate))</definedName>
+    <definedName name="TAX_SE">_xlfn.LAMBDA(se_net_earnings,year,_xlfn.LET(se_base,se_net_earnings*0.9235,ss_cap,INDEX(_xlfn._xlws.FILTER(tblThresholds[Value],(tblThresholds[Item]="SS_Wage_Base")*(tblThresholds[Year]=year)),1),ss_tax,MIN(se_base,ss_cap)*0.124,medi_tax,se_base*0.029,ss_tax+medi_tax))</definedName>
+    <definedName name="STD_DED">_xlfn.LAMBDA(year,fs,INDEX(_xlfn._xlws.FILTER(tblStdDed[Amount],(tblStdDed[Year]=year)*(tblStdDed[FilingStatus]=fs)),1))</definedName>
+    <definedName name="TAX_STATE">_xlfn.LAMBDA(taxable_income,state,taxable_income*_xlfn.XLOOKUP(state,tblStateRates[State],tblStateRates[Top_Marginal_Rate],0))</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
   <pivotCaches>
@@ -2783,7 +2783,21 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tblMasterStrategies" displayName="tblMasterStrategies" ref="B7:L26" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="tblStateRates" displayName="tblStateRates" ref="B618:F669" headerRowCount="1">
+  <autoFilter ref="B618:F669"/>
+  <tableColumns count="5">
+    <tableColumn id="2" name="State"/>
+    <tableColumn id="3" name="Top_Marginal_Rate"/>
+    <tableColumn id="4" name="Has_PTET"/>
+    <tableColumn id="5" name="PTET_Rate"/>
+    <tableColumn id="6" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tblMasterStrategies" displayName="tblMasterStrategies" ref="B7:L26" headerRowCount="1">
   <autoFilter ref="B7:L26"/>
   <tableColumns count="11">
     <tableColumn id="2" name="Strategy_ID"/>
@@ -26732,7 +26746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J669"/>
+  <dimension ref="B2:J670"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="3.6328125" customWidth="1" style="99" min="1" max="1"/>
@@ -39250,6 +39264,7 @@
         </is>
       </c>
     </row>
+    <row r="617"/>
     <row r="618">
       <c r="B618" s="145" t="inlineStr">
         <is>
@@ -40422,18 +40437,20 @@
         </is>
       </c>
     </row>
+    <row r="670"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B616:I616"/>
     <mergeCell ref="B615:I615"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="5">
+  <tableParts count="6">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>